<commit_message>
auto: scan 2026-05-23 13:20 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -437,7 +437,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>$10000.00</t>
+          <t>$9604.00</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,79 +519,218 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>market_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>market_title</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>team_a</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>team_b</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>fill_price</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>size</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>model_prob</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>market_prob</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>edge</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>opened_at</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>resolution_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>pnl</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>outcome</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>a99a57ee</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2269581</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>LoL: DN SOOPers vs Gen.G (BO3) - LCK Rounds 1-2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DN SOOPers</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Gen.G</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.042581</v>
+      </c>
+      <c r="H2" t="n">
+        <v>200</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.2917631023100087</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0405</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.2512631023100087</v>
+      </c>
+      <c r="L2" t="n">
+        <v>76</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-05-23T10:39:26.839437+00:00</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-05-24T14:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>7a945880</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2293225</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LoL: LYON vs Team Liquid (BO5) - LCS Playoffs</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LYON</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.014525</v>
+      </c>
+      <c r="H3" t="n">
+        <v>196</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.4112154962256769</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.3987154962256769</v>
+      </c>
+      <c r="L3" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-05-23T10:39:26.841498+00:00</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-05-25T01:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto: scan 2026-05-24 12:24 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -437,7 +437,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>$9604.00</t>
+          <t>$9507.96</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,6 +732,73 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>8b27c31c</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2293200</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>LoL: LYON vs Team Liquid (BO5) - LCS Playoffs</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LYON</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.45791</v>
+      </c>
+      <c r="H4" t="n">
+        <v>96.04000000000001</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5887845037743231</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1337845037743231</v>
+      </c>
+      <c r="L4" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-05-24T12:24:54.276876+00:00</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-05-25T02:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add 14:30 and 22:00 UTC resolve slots for LCK/LEC match times
09:30 UTC resolve only covered early LPL games.
LCK afternoon games resolve ~14:00 UTC, LEC/LCS ~21:00-22:00 UTC.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,12 +430,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -512,87 +524,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>market_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>market_title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>team_a</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>team_b</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fill_price</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>size</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>model_prob</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>market_prob</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>edge</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>opened_at</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>resolution_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>pnl</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>outcome</t>
         </is>
@@ -735,51 +747,51 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8b27c31c</t>
+          <t>d7f1738b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2293200</t>
+          <t>2342527</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LoL: LYON vs Team Liquid (BO5) - LCS Playoffs</t>
+          <t>LoL: DN SOOPers vs Nongshim Red Force (BO3) - LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LYON</t>
+          <t>DN SOOPers</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>Nongshim RedForce</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BUY_NO</t>
+          <t>BUY_YES</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.45791</v>
+        <v>0.24248</v>
       </c>
       <c r="H4" t="n">
         <v>96.04000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>0.5887845037743231</v>
+        <v>0.6400862102361262</v>
       </c>
       <c r="J4" t="n">
-        <v>0.455</v>
+        <v>0.24</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1337845037743231</v>
+        <v>0.4000862102361262</v>
       </c>
       <c r="L4" t="n">
-        <v>67.90000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -788,12 +800,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-24T12:24:54.276876+00:00</t>
+          <t>2026-05-24T12:13:19.544607+00:00</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-25T02:00:00+00:00</t>
+          <t>2026-05-28T14:00:00+00:00</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>

</xml_diff>

<commit_message>
auto: scan 2026-05-24 13:23 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,12 +418,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -524,87 +512,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>market_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>market_title</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>team_a</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>team_b</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>fill_price</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>size</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>model_prob</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>market_prob</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>edge</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>opened_at</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>resolution_date</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>pnl</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>outcome</t>
         </is>

</xml_diff>

<commit_message>
auto: scan 2026-05-25 04:55 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -414,8 +414,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -432,69 +436,105 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Generated At</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>$9507.96</t>
+          <t>2026-05-25 04:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Portfolio Value</t>
+          <t>Starting Capital</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>$10000.00</t>
+          <t>$10,000.00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Total PnL</t>
+          <t>Current Capital</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$0.00</t>
+          <t>$9507.96</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Win Rate</t>
+          <t>Portfolio Value</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>$10000.00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total Trades</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
+          <t>Total PnL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$+0.00</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Win Rate</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Resolved Trades</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Open Positions</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Avg Edge (resolved)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -508,296 +548,282 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Match</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>market_id</t>
+          <t>Tournament</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>market_title</t>
+          <t>Bet</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>team_a</t>
+          <t>Size ($)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>team_b</t>
+          <t>Fill Price</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>Model Prob</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>fill_price</t>
+          <t>Market Prob</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>size</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>model_prob</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>market_prob</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>edge</t>
+          <t>Outcome</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>PnL ($)</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Opened</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>opened_at</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>resolution_date</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>pnl</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>outcome</t>
+          <t>Resolves</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>a99a57ee</t>
+          <t>DN SOOPers vs Gen.G</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2269581</t>
+          <t>LoL: DN SOOPers vs Gen.G (BO3) - LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LoL: DN SOOPers vs Gen.G (BO3) - LCK Rounds 1-2</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DN SOOPers</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Gen.G</t>
-        </is>
+          <t>Bet DN SOOPers to win</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>200</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0426</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BUY_YES</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>0.042581</v>
-      </c>
-      <c r="H2" t="n">
-        <v>200</v>
+          <t>29.2%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>4.0%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>+25.1%</t>
+        </is>
       </c>
       <c r="I2" t="n">
-        <v>0.2917631023100087</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.0405</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.2512631023100087</v>
-      </c>
-      <c r="L2" t="n">
         <v>76</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>2026-05-23 10:39</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-23T10:39:26.839437+00:00</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>2026-05-24T14:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+          <t>2026-05-24 14:00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7a945880</t>
+          <t>LYON vs TL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2293225</t>
+          <t>LoL: LYON vs Team Liquid (BO5) - LCS Playoffs</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LoL: LYON vs Team Liquid (BO5) - LCS Playoffs</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LYON</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
+          <t>Bet LYON to win</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>196</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0145</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>BUY_YES</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>0.014525</v>
-      </c>
-      <c r="H3" t="n">
-        <v>196</v>
+          <t>41.1%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1.2%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>+39.9%</t>
+        </is>
       </c>
       <c r="I3" t="n">
-        <v>0.4112154962256769</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.0125</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.3987154962256769</v>
-      </c>
-      <c r="L3" t="n">
         <v>64.7</v>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>2026-05-23 10:39</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-23T10:39:26.841498+00:00</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>2026-05-25T01:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+          <t>2026-05-25 01:00</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>d7f1738b</t>
+          <t>DN SOOPers vs Nongshim RedForce</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2342527</t>
+          <t>LoL: DN SOOPers vs Nongshim Red Force (BO3) - LCK Rounds 1-2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LoL: DN SOOPers vs Nongshim Red Force (BO3) - LCK Rounds 1-2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DN SOOPers</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Nongshim RedForce</t>
-        </is>
+          <t>Bet DN SOOPers to win</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>96.04000000000001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.2425</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BUY_YES</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>0.24248</v>
-      </c>
-      <c r="H4" t="n">
-        <v>96.04000000000001</v>
+          <t>64.0%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>24.0%</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>+40.0%</t>
+        </is>
       </c>
       <c r="I4" t="n">
-        <v>0.6400862102361262</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.4000862102361262</v>
-      </c>
-      <c r="L4" t="n">
         <v>68.5</v>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>2026-05-24 12:13</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-24T12:13:19.544607+00:00</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>2026-05-28T14:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+          <t>2026-05-28 14:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto: resolve 2026-05-28 12:48 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 09:42 UTC</t>
+          <t>2026-05-28 12:48 UTC</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$10000.00</t>
+          <t>$9604.00</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$+0.00</t>
+          <t>$-396.00</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -533,7 +533,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+32.5%</t>
         </is>
       </c>
     </row>
@@ -560,8 +560,8 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
@@ -681,15 +681,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+          <t>LOSS — Gen.G won</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>-200</v>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>2026-05-23 10:39</t>
@@ -743,15 +745,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
+          <t>LOSS — TL won</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>-196</v>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>2026-05-23 10:39</t>

</xml_diff>

<commit_message>
auto: scan 2026-05-28 15:47 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 12:48 UTC</t>
+          <t>2026-05-28 15:47 UTC</t>
         </is>
       </c>
     </row>
@@ -465,7 +465,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$9507.96</t>
+          <t>$9412.88</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -829,6 +829,68 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TES vs LGD Gaming</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LoL: Top Esports vs LGD Gaming (BO5) - LPL Playoffs</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bet LGD Gaming to win</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>95.08</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>36.3%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>+20.8%</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-28 15:47</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-05-29 15:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: resolve 2026-05-28 17:48 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 15:47 UTC</t>
+          <t>2026-05-28 17:48 UTC</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$9604.00</t>
+          <t>$9507.96</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$-396.00</t>
+          <t>$-492.04</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -533,7 +533,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>+32.5%</t>
+          <t>+35.0%</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
@@ -809,15 +809,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
+          <t>LOSS — Nongshim RedForce won</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>-96.04000000000001</v>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t>2026-05-24 12:13</t>

</xml_diff>

<commit_message>
auto: scan 2026-05-28 20:03 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 17:48 UTC</t>
+          <t>2026-05-28 20:03 UTC</t>
         </is>
       </c>
     </row>
@@ -465,7 +465,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$9412.88</t>
+          <t>$9225.56</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -548,12 +548,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -893,6 +893,130 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TES vs LGD Gaming</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LoL: Top Esports vs LGD Gaming (BO5) - LPL Playoffs</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bet LGD Gaming to win</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>94.13</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>36.3%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>+20.8%</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-28 20:03</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-05-29 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TL vs Shopify Rebellion</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LoL: Team Liquid vs Shopify Rebellion (BO5) - LCS Playoffs</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Bet Shopify Rebellion to win</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>93.19</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>40.2%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>+24.7%</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-28 20:03</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-06-01 02:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: resolve 2026-05-29 17:48 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-29 14:58 UTC</t>
+          <t>2026-05-29 17:48 UTC</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$9507.96</t>
+          <t>$9318.75</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$-492.04</t>
+          <t>$-681.25</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -533,7 +533,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>+35.0%</t>
+          <t>+29.3%</t>
         </is>
       </c>
     </row>
@@ -873,15 +873,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
+          <t>LOSS — TES won</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>-95.08</v>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
           <t>2026-05-28 15:47</t>
@@ -935,15 +937,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
+          <t>LOSS — TES won</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>-94.13</v>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
           <t>2026-05-28 20:03</t>

</xml_diff>

<commit_message>
auto: scan 2026-05-29 20:04 UTC
</commit_message>
<xml_diff>
--- a/exports/esports_report.xlsx
+++ b/exports/esports_report.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-29 17:48 UTC</t>
+          <t>2026-05-29 20:04 UTC</t>
         </is>
       </c>
     </row>
@@ -465,7 +465,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$9225.56</t>
+          <t>$9041.97</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1021,6 +1021,130 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BLG vs Team WE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LoL: Bilibili Gaming vs Team WE (BO5) - LPL Playoffs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bet BLG to win</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>92.26000000000001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5481</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>70.4%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>54.5%</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>+15.9%</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-29 20:04</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-05-30 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TL vs Shopify Rebellion</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LoL: Team Liquid vs Shopify Rebellion (BO5) - LCS Playoffs</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Bet Shopify Rebellion to win</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>91.33</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>40.2%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>+24.7%</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-29 20:04</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-06-01 02:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>